<commit_message>
correction erreurs fr 1
</commit_message>
<xml_diff>
--- a/Data_communes/divisions_tableau.xlsx
+++ b/Data_communes/divisions_tableau.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="45" windowWidth="28455" windowHeight="12540"/>
+    <workbookView xWindow="240" yWindow="48" windowWidth="23256" windowHeight="12540"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -19,14 +19,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="46">
   <si>
     <t>01 - Produits alimentaires et boissons non alcoolisées</t>
   </si>
   <si>
-    <t>04 - Logement, eau, gaz, électricité et autres combustibles</t>
-  </si>
-  <si>
     <t>05 - Meubles, articles de ménages et entretien courant du foyer</t>
   </si>
   <si>
@@ -55,9 +52,6 @@
   </si>
   <si>
     <t>06 – Santé</t>
-  </si>
-  <si>
-    <t>07 – Transport</t>
   </si>
   <si>
     <t>08 – Communications</t>
@@ -137,24 +131,12 @@
     <t>01 – Food products and non-alcoholic</t>
   </si>
   <si>
-    <t>02 –Alcoholicbeverages and tobacco</t>
-  </si>
-  <si>
-    <t>Non foodproducts</t>
-  </si>
-  <si>
     <t>03 – Clothing and shoes</t>
   </si>
   <si>
-    <t>04 - Housing, water, gas, electricity and other fuel</t>
-  </si>
-  <si>
     <t>06 –Health</t>
   </si>
   <si>
-    <t>08 – Communication</t>
-  </si>
-  <si>
     <t>09 – Leisure and culture</t>
   </si>
   <si>
@@ -164,20 +146,35 @@
     <t>11 - Restaurants and hotels</t>
   </si>
   <si>
-    <t>12 – Variousgoods and services</t>
-  </si>
-  <si>
     <t>General index</t>
   </si>
   <si>
     <t>05 - Furniture, household items and routine maintenance of the home</t>
+  </si>
+  <si>
+    <t>07 – Transports</t>
+  </si>
+  <si>
+    <t>04 - Logement, eau, électricité, gaz et autres combustibles</t>
+  </si>
+  <si>
+    <t>04 - Housing, water, electricity, gas and other fuel</t>
+  </si>
+  <si>
+    <t>02 –Alcoholic beverages and tobacco</t>
+  </si>
+  <si>
+    <t>Non food products</t>
+  </si>
+  <si>
+    <t>12 – Various goods and services</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -202,6 +199,12 @@
       <color rgb="FF000000"/>
       <name val="ArabicTypesetting"/>
     </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FFFF0000"/>
+      <name val="TimesNewRomanPS-BoldMT"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -223,13 +226,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" readingOrder="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -526,187 +543,187 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="59.140625" customWidth="1"/>
-    <col min="2" max="2" width="46.28515625" customWidth="1"/>
-    <col min="3" max="3" width="34.42578125" style="4" customWidth="1"/>
+    <col min="1" max="1" width="59.109375" customWidth="1"/>
+    <col min="2" max="2" width="46.33203125" customWidth="1"/>
+    <col min="3" max="3" width="34.44140625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" s="2" t="s">
         <v>5</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>33</v>
+        <v>6</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>34</v>
+      <c r="B3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>35</v>
+        <v>7</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>36</v>
+        <v>8</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="21.6">
+      <c r="A8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="22.5">
-      <c r="A7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="22.5">
-      <c r="A8" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>46</v>
+      <c r="C8" s="2" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>25</v>
+        <v>10</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>23</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:3">
-      <c r="A10" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>12</v>
+      <c r="A10" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>40</v>
+        <v>11</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>28</v>
+        <v>12</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>26</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>29</v>
+        <v>13</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>27</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>30</v>
+        <v>14</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>28</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>44</v>
+        <v>15</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>32</v>
+        <v>2</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>30</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -718,7 +735,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -727,7 +744,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>